<commit_message>
HubBoard C0 updates: system power is controlled via a slide switch
</commit_message>
<xml_diff>
--- a/SensWear-V1R1-Main/Output/Manufacturing/Assembly/Bill of Materials/Bill of Materials-SensWear-V1R1-MainBoard.xlsx
+++ b/SensWear-V1R1-Main/Output/Manufacturing/Assembly/Bill of Materials/Bill of Materials-SensWear-V1R1-MainBoard.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORK\Projects\OpenRing\Hardware\SensWear-V1R1-Main\Output\Manufacturing\Assembly\Bill of Materials\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORK\Projects\SensWear\hardware-v1\SensWear-V1R1-Main\Output\Manufacturing\Assembly\Bill of Materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7AB2388D-7BF8-4EDF-BCC4-F089DBD8151A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{453EE4DF-BDDB-402B-AD66-025AAFAEF3DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{07270503-5351-47F7-9BC7-9D25E3D2FE9D}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="28800" windowHeight="17170" xr2:uid="{8CE0689D-23DE-4210-B178-6762B10BE0B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-SensWear-V1R1" sheetId="1" r:id="rId1"/>
@@ -34,12 +34,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="215">
   <si>
     <t>Manufacturer</t>
   </si>
@@ -56,7 +59,7 @@
     <t>Value</t>
   </si>
   <si>
-    <t>Comment</t>
+    <t>Name</t>
   </si>
   <si>
     <t>Description</t>
@@ -254,6 +257,18 @@
     <t>1276-CL10A476MQ8QRNCCT-ND</t>
   </si>
   <si>
+    <t>CSD75207W15</t>
+  </si>
+  <si>
+    <t>T1</t>
+  </si>
+  <si>
+    <t>MOSFET 2P-CH 3.9A 9DSBGA</t>
+  </si>
+  <si>
+    <t>Arrow Electronics</t>
+  </si>
+  <si>
     <t>DFE201612E-2R2M=P2</t>
   </si>
   <si>
@@ -269,6 +284,21 @@
     <t>81-DFE201612E-2R2MP2</t>
   </si>
   <si>
+    <t>Panasonic</t>
+  </si>
+  <si>
+    <t>ERJ2RKF2202X</t>
+  </si>
+  <si>
+    <t>R5</t>
+  </si>
+  <si>
+    <t>22kΩ</t>
+  </si>
+  <si>
+    <t>Res Thick Film 0402 22K Ohm 1% 0.1W(1/10W) ±100ppm/C Pad SMD Automotive T/R</t>
+  </si>
+  <si>
     <t>Panasonic Electronic Components</t>
   </si>
   <si>
@@ -320,7 +350,7 @@
     <t>ERJ-2RKF1004X</t>
   </si>
   <si>
-    <t>R1, R3, R6, R7, R8, R9</t>
+    <t>R1, R3, R6, R7, R8, R9, R10</t>
   </si>
   <si>
     <t>1 M</t>
@@ -615,6 +645,24 @@
   </si>
   <si>
     <t>LED Low-Power Tri-Color Blue/Green/Red 465nm/518nm/632nm 2.7V/2.75V/1.95V 4-Pin SMD T/R</t>
+  </si>
+  <si>
+    <t>ALPS</t>
+  </si>
+  <si>
+    <t>SSAJ110100</t>
+  </si>
+  <si>
+    <t>SW1</t>
+  </si>
+  <si>
+    <t>Slide Switch, SPDT, Latched, 0.01A, 5VDC, Solder Terminal, Surface Mount-right Angle</t>
+  </si>
+  <si>
+    <t>DigiKey</t>
+  </si>
+  <si>
+    <t>4809-SSAJ110100DKR-ND</t>
   </si>
   <si>
     <t>TPS62840YBGR</t>
@@ -1034,22 +1082,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{634643FE-CF66-493D-ACC4-FAFAB62CB7CA}">
-  <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA076C61-DBD8-41D1-A7D0-9748EA871FA5}">
+  <dimension ref="A1:I42"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" customWidth="1"/>
-    <col min="2" max="2" width="23.140625" customWidth="1"/>
-    <col min="3" max="3" width="30.85546875" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" customWidth="1"/>
-    <col min="5" max="5" width="16.5703125" customWidth="1"/>
-    <col min="6" max="6" width="25.42578125" customWidth="1"/>
-    <col min="7" max="7" width="105" customWidth="1"/>
-    <col min="8" max="8" width="18.85546875" customWidth="1"/>
-    <col min="9" max="9" width="27" customWidth="1"/>
+    <col min="1" max="1" width="15.81640625" customWidth="1"/>
+    <col min="2" max="2" width="22.1796875" customWidth="1"/>
+    <col min="3" max="3" width="29.6328125" customWidth="1"/>
+    <col min="4" max="4" width="9.453125" customWidth="1"/>
+    <col min="5" max="5" width="15.81640625" customWidth="1"/>
+    <col min="6" max="6" width="24.26953125" customWidth="1"/>
+    <col min="7" max="7" width="100.7265625" customWidth="1"/>
+    <col min="8" max="8" width="18.08984375" customWidth="1"/>
+    <col min="9" max="9" width="25.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1078,7 +1126,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="2" t="s">
@@ -1097,7 +1145,7 @@
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1124,7 +1172,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>18</v>
       </c>
@@ -1151,7 +1199,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -1178,7 +1226,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>27</v>
       </c>
@@ -1205,7 +1253,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>33</v>
       </c>
@@ -1232,7 +1280,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>40</v>
       </c>
@@ -1259,7 +1307,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>46</v>
       </c>
@@ -1286,7 +1334,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>51</v>
       </c>
@@ -1313,7 +1361,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>51</v>
       </c>
@@ -1340,7 +1388,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>60</v>
       </c>
@@ -1369,7 +1417,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>60</v>
       </c>
@@ -1398,9 +1446,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>71</v>
@@ -1411,645 +1459,651 @@
       <c r="D14" s="1">
         <v>1</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="1"/>
+      <c r="F14" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="G14" s="2" t="s">
+      <c r="H14" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="I14" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D15" s="1">
+        <v>1</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="H15" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D15" s="1">
+      <c r="I15" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D16" s="1">
+        <v>1</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D17" s="1">
         <v>2</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D16" s="1">
-        <v>1</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C17" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D17" s="1">
-        <v>1</v>
-      </c>
-      <c r="E17" s="2" t="s">
+      <c r="F17" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>90</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>38</v>
       </c>
       <c r="I17" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="1">
+        <v>1</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D18" s="1">
-        <v>6</v>
-      </c>
-      <c r="E18" s="2" t="s">
+      <c r="F18" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>95</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>38</v>
       </c>
       <c r="I18" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="1">
+        <v>1</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D19" s="1">
-        <v>3</v>
-      </c>
-      <c r="E19" s="2" t="s">
+      <c r="F19" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>38</v>
       </c>
       <c r="I19" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B20" s="2" t="s">
+      <c r="C20" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="D20" s="1">
+        <v>7</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D20" s="1">
-        <v>1</v>
-      </c>
-      <c r="E20" s="2" t="s">
+      <c r="F20" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="F20" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="G20" s="2" t="s">
+      <c r="H20" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I20" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="H20" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I20" s="2" t="s">
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="D21" s="1">
+        <v>3</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="D21" s="1">
-        <v>1</v>
-      </c>
-      <c r="E21" s="2" t="s">
+      <c r="F21" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G21" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="F21" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="G21" s="2" t="s">
+      <c r="H21" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I21" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="H21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>46</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="1">
+        <v>1</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D22" s="1">
-        <v>1</v>
-      </c>
-      <c r="E22" s="2" t="s">
+      <c r="F22" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>115</v>
       </c>
       <c r="H22" s="2" t="s">
         <v>16</v>
       </c>
       <c r="I22" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
+      <c r="C23" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="D23" s="1">
+        <v>1</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="F23" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G23" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="D23" s="1">
+      <c r="H23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D24" s="1">
+        <v>1</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D25" s="1">
         <v>2</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="H23" s="2" t="s">
+      <c r="E25" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="H25" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I23" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="D24" s="1">
+      <c r="I25" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D26" s="1">
         <v>3</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="H24" s="2" t="s">
+      <c r="E26" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="H26" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I24" s="2" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="D25" s="1">
-        <v>5</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I25" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="D26" s="1">
-        <v>10</v>
-      </c>
-      <c r="E26" s="2" t="s">
+      <c r="I26" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F26" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>46</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D27" s="1">
+        <v>5</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="F27" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="G27" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="D27" s="1">
-        <v>1</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>142</v>
       </c>
       <c r="H27" s="2" t="s">
         <v>16</v>
       </c>
       <c r="I27" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B28" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="D28" s="1">
+        <v>10</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D28" s="1">
-        <v>3</v>
-      </c>
-      <c r="E28" s="2" t="s">
+      <c r="F28" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="G28" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="F28" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="G28" s="2" t="s">
+      <c r="H28" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I28" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="H28" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>46</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="D29" s="1">
+        <v>1</v>
+      </c>
+      <c r="E29" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="D29" s="1">
-        <v>2</v>
-      </c>
-      <c r="E29" s="2" t="s">
+      <c r="F29" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="G29" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>152</v>
       </c>
       <c r="H29" s="2" t="s">
         <v>16</v>
       </c>
       <c r="I29" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B30" s="2" t="s">
+      <c r="C30" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="D30" s="1">
+        <v>3</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="D30" s="1">
-        <v>1</v>
-      </c>
-      <c r="E30" s="1"/>
       <c r="F30" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="G30" s="2" t="s">
         <v>156</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>157</v>
       </c>
       <c r="H30" s="2" t="s">
         <v>38</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>46</v>
       </c>
       <c r="B31" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="D31" s="1">
+        <v>2</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="D31" s="1">
-        <v>1</v>
-      </c>
-      <c r="E31" s="2" t="s">
+      <c r="F31" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="G31" s="2" t="s">
         <v>161</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>162</v>
       </c>
       <c r="H31" s="2" t="s">
         <v>16</v>
       </c>
       <c r="I31" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B32" s="2" t="s">
+      <c r="C32" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="D32" s="1">
+        <v>1</v>
+      </c>
+      <c r="E32" s="1"/>
+      <c r="F32" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="D32" s="1">
-        <v>2</v>
-      </c>
-      <c r="E32" s="2" t="s">
+      <c r="G32" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="F32" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="G32" s="2" t="s">
+      <c r="H32" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I32" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="H32" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I32" s="2" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>46</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="D33" s="1">
+        <v>1</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="D33" s="1">
-        <v>1</v>
-      </c>
-      <c r="E33" s="2" t="s">
+      <c r="F33" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="G33" s="2" t="s">
         <v>171</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>172</v>
       </c>
       <c r="H33" s="2" t="s">
         <v>16</v>
       </c>
       <c r="I33" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="D34" s="1">
+        <v>2</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="C34" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="D34" s="1">
-        <v>1</v>
-      </c>
-      <c r="E34" s="1"/>
       <c r="F34" s="2" t="s">
         <v>175</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>16</v>
       </c>
       <c r="I34" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
+      <c r="C35" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="D35" s="1">
+        <v>1</v>
+      </c>
+      <c r="E35" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="F35" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="G35" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="D35" s="1">
-        <v>1</v>
-      </c>
-      <c r="E35" s="1"/>
-      <c r="F35" s="2" t="s">
+      <c r="H35" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I35" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="G35" s="2" t="s">
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A36" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="H35" s="1"/>
-      <c r="I35" s="1"/>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="2" t="s">
+      <c r="B36" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>185</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>186</v>
       </c>
       <c r="D36" s="1">
         <v>1</v>
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G36" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I36" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="H36" s="1"/>
-      <c r="I36" s="1"/>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>188</v>
       </c>
@@ -2064,66 +2118,139 @@
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="2" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>51</v>
+        <v>193</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D38" s="1">
         <v>1</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I38" s="2" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+        <v>196</v>
+      </c>
+      <c r="H38" s="1"/>
+      <c r="I38" s="1"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
-        <v>51</v>
+        <v>197</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D39" s="1">
         <v>1</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="H39" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="H39" s="1"/>
+      <c r="I39" s="1"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D40" s="1">
+        <v>1</v>
+      </c>
+      <c r="E40" s="1"/>
+      <c r="F40" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A41" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="D41" s="1">
+        <v>1</v>
+      </c>
+      <c r="E41" s="1"/>
+      <c r="F41" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H41" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="I39" s="2" t="s">
-        <v>199</v>
+      <c r="I41" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="D42" s="1">
+        <v>1</v>
+      </c>
+      <c r="E42" s="1"/>
+      <c r="F42" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
inductor update triggered updated outputs
</commit_message>
<xml_diff>
--- a/SensWear-V1R1-Main/Output/Manufacturing/Assembly/Bill of Materials/Bill of Materials-SensWear-V1R1-MainBoard.xlsx
+++ b/SensWear-V1R1-Main/Output/Manufacturing/Assembly/Bill of Materials/Bill of Materials-SensWear-V1R1-MainBoard.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORK\Projects\SensWear\hardware-v1\SensWear-V1R1-Main\Output\Manufacturing\Assembly\Bill of Materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{453EE4DF-BDDB-402B-AD66-025AAFAEF3DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{89FC18F1-8853-4EB5-9BF9-F54FCCBE6FD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="28800" windowHeight="17170" xr2:uid="{8CE0689D-23DE-4210-B178-6762B10BE0B3}"/>
+    <workbookView xWindow="4290" yWindow="4290" windowWidth="28800" windowHeight="15345" xr2:uid="{4A779FA2-59A9-4371-9698-68B29AD8918D}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-SensWear-V1R1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="216">
   <si>
     <t>Manufacturer</t>
   </si>
@@ -578,49 +578,52 @@
     <t>81-LQG15WH3N5B02D</t>
   </si>
   <si>
-    <t>LQM18FN4R7M00D</t>
+    <t>STMicroelectronics</t>
+  </si>
+  <si>
+    <t>M95P32-IXCST/EF</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>M95P32-I Series 32 Mb (4 M x 8) 80 MHz SPI EEPROM Memory IC - WLCSP-8</t>
+  </si>
+  <si>
+    <t>511-M95P32-IXCST/EF</t>
+  </si>
+  <si>
+    <t>Nordic Semiconductor</t>
+  </si>
+  <si>
+    <t>NRF54L15-QFAA-R</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>NRF54L15-QF</t>
+  </si>
+  <si>
+    <t>nRF54L15 SoC with Arm Cortex-M33 processor</t>
+  </si>
+  <si>
+    <t>TDK</t>
+  </si>
+  <si>
+    <t>PLEA67BCA4R7M-1PT00</t>
   </si>
   <si>
     <t>L3</t>
   </si>
   <si>
-    <t>4.7uH</t>
-  </si>
-  <si>
-    <t>Inductor Power Chip Shielded Multi-Layer 4.7uH 20% 1MHz Ferrite 0.08A 0.78Ohm DCR 0603 T/R</t>
-  </si>
-  <si>
-    <t>81-LQM18FN4R7M00D</t>
-  </si>
-  <si>
-    <t>STMicroelectronics</t>
-  </si>
-  <si>
-    <t>M95P32-IXCST/EF</t>
-  </si>
-  <si>
-    <t>U2</t>
-  </si>
-  <si>
-    <t>M95P32-I Series 32 Mb (4 M x 8) 80 MHz SPI EEPROM Memory IC - WLCSP-8</t>
-  </si>
-  <si>
-    <t>511-M95P32-IXCST/EF</t>
-  </si>
-  <si>
-    <t>Nordic Semiconductor</t>
-  </si>
-  <si>
-    <t>NRF54L15-QFAA-R</t>
-  </si>
-  <si>
-    <t>U1</t>
-  </si>
-  <si>
-    <t>NRF54L15-QF</t>
-  </si>
-  <si>
-    <t>nRF54L15 SoC with Arm Cortex-M33 processor</t>
+    <t>4.7µH</t>
+  </si>
+  <si>
+    <t>1MHz 300mA 300mA 4.7μH 1.08Ω ±20% 0402 SMD mount 1.1mm(Length)*800μm(height)</t>
+  </si>
+  <si>
+    <t>Farnell</t>
   </si>
   <si>
     <t>XTPogoPin</t>
@@ -1082,22 +1085,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA076C61-DBD8-41D1-A7D0-9748EA871FA5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AD6BFA6-A86E-4EF2-8F26-B5A15A637D58}">
   <dimension ref="A1:I42"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.81640625" customWidth="1"/>
-    <col min="2" max="2" width="22.1796875" customWidth="1"/>
-    <col min="3" max="3" width="29.6328125" customWidth="1"/>
-    <col min="4" max="4" width="9.453125" customWidth="1"/>
-    <col min="5" max="5" width="15.81640625" customWidth="1"/>
-    <col min="6" max="6" width="24.26953125" customWidth="1"/>
-    <col min="7" max="7" width="100.7265625" customWidth="1"/>
-    <col min="8" max="8" width="18.08984375" customWidth="1"/>
-    <col min="9" max="9" width="25.81640625" customWidth="1"/>
+    <col min="1" max="1" width="16.5703125" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" customWidth="1"/>
+    <col min="3" max="3" width="30.85546875" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" customWidth="1"/>
+    <col min="6" max="6" width="25.42578125" customWidth="1"/>
+    <col min="7" max="7" width="105" customWidth="1"/>
+    <col min="8" max="8" width="18.85546875" customWidth="1"/>
+    <col min="9" max="9" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1126,7 +1129,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="2" t="s">
@@ -1145,7 +1148,7 @@
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1172,7 +1175,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>18</v>
       </c>
@@ -1199,7 +1202,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -1226,7 +1229,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>27</v>
       </c>
@@ -1253,7 +1256,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>33</v>
       </c>
@@ -1280,7 +1283,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>40</v>
       </c>
@@ -1307,7 +1310,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>46</v>
       </c>
@@ -1334,7 +1337,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>51</v>
       </c>
@@ -1361,7 +1364,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>51</v>
       </c>
@@ -1388,7 +1391,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>60</v>
       </c>
@@ -1417,7 +1420,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>60</v>
       </c>
@@ -1446,7 +1449,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>51</v>
       </c>
@@ -1473,7 +1476,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>46</v>
       </c>
@@ -1502,7 +1505,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>80</v>
       </c>
@@ -1527,7 +1530,7 @@
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>85</v>
       </c>
@@ -1556,7 +1559,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>85</v>
       </c>
@@ -1585,7 +1588,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>85</v>
       </c>
@@ -1614,7 +1617,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>85</v>
       </c>
@@ -1643,7 +1646,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>85</v>
       </c>
@@ -1672,7 +1675,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>46</v>
       </c>
@@ -1701,7 +1704,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>46</v>
       </c>
@@ -1730,7 +1733,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>46</v>
       </c>
@@ -1759,7 +1762,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>126</v>
       </c>
@@ -1788,7 +1791,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>126</v>
       </c>
@@ -1817,7 +1820,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>46</v>
       </c>
@@ -1846,7 +1849,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>142</v>
       </c>
@@ -1875,7 +1878,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>46</v>
       </c>
@@ -1904,7 +1907,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>126</v>
       </c>
@@ -1933,7 +1936,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>46</v>
       </c>
@@ -1962,7 +1965,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>51</v>
       </c>
@@ -1989,7 +1992,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>46</v>
       </c>
@@ -2018,7 +2021,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>46</v>
       </c>
@@ -2047,24 +2050,22 @@
         <v>177</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>46</v>
+        <v>178</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C35" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D35" s="1">
+        <v>1</v>
+      </c>
+      <c r="E35" s="1"/>
+      <c r="F35" s="2" t="s">
         <v>179</v>
-      </c>
-      <c r="D35" s="1">
-        <v>1</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>180</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>181</v>
@@ -2076,7 +2077,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>183</v>
       </c>
@@ -2091,19 +2092,15 @@
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I36" s="2" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H36" s="1"/>
+      <c r="I36" s="1"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>188</v>
       </c>
@@ -2116,141 +2113,147 @@
       <c r="D37" s="1">
         <v>1</v>
       </c>
-      <c r="E37" s="1"/>
+      <c r="E37" s="2" t="s">
+        <v>191</v>
+      </c>
       <c r="F37" s="2" t="s">
         <v>191</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="H37" s="1"/>
-      <c r="I37" s="1"/>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H37" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D38" s="1">
         <v>1</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D39" s="1">
         <v>1</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D40" s="1">
         <v>1</v>
       </c>
       <c r="E40" s="1"/>
       <c r="F40" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>51</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D41" s="1">
         <v>1</v>
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="H41" s="2" t="s">
         <v>16</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>51</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D42" s="1">
         <v>1</v>
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>16</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>

</xml_diff>